<commit_message>
feat: implement scenario utilities and master visualizer while generating comprehensive optimization model results and MCDM analysis files
</commit_message>
<xml_diff>
--- a/data/scenarios/scenarios.xlsx
+++ b/data/scenarios/scenarios.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -437,11 +437,6 @@
           <t>Q_i</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Q_i_file</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -456,13 +451,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Yol kapanmasi yok. Q_i=1.0.</t>
+          <t>Yol kapanmasi yok (Q_i=1.0). Standart MCLP/MILP problemi.</t>
         </is>
       </c>
       <c r="D2" t="n">
         <v>1</v>
       </c>
-      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -477,15 +471,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>mu_ij_eff = mu_ij * Q_i (gercek p_road_open). Lokal konumlanmayi tesvik eder.</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>results/fcm/Q_i_vector.xlsx</t>
+          <t>mu_ij_eff = mu_ij * Q_i. Yol kapanmasi uzak konteynerlerin etkisini azaltir, lokal konumlanmayi one cikarir.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>gercek</t>
         </is>
       </c>
     </row>

</xml_diff>